<commit_message>
Deploying to main from @ open-resource-discovery/specification@55caeca83ed2c004a1f2e534fd386355458b7738 🚀
</commit_message>
<xml_diff>
--- a/specification/pr-202/spec-v1/interfaces/Document.xlsx
+++ b/specification/pr-202/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1462" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1471" uniqueCount="209">
   <si>
     <t>Entity Name</t>
   </si>
@@ -482,6 +482,15 @@
   </si>
   <si>
     <t>Capability Integration Aspect</t>
+  </si>
+  <si>
+    <t>array&lt;CapabilityIntegrationAspectSubset&gt;</t>
+  </si>
+  <si>
+    <t>Capability Integration Aspect Subset</t>
+  </si>
+  <si>
+    <t>skillName</t>
   </si>
   <si>
     <t>Vendor</t>
@@ -1005,7 +1014,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D487"/>
+  <dimension ref="A1:D490"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5437,13 +5446,13 @@
         <v>127</v>
       </c>
       <c r="B317" t="s">
-        <v>94</v>
+        <v>121</v>
       </c>
       <c r="C317" t="b">
         <v>0</v>
       </c>
       <c r="D317" t="s">
-        <v>130</v>
+        <v>9</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.25">
@@ -5451,13 +5460,13 @@
         <v>127</v>
       </c>
       <c r="B318" t="s">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="C318" t="b">
         <v>0</v>
       </c>
       <c r="D318" t="s">
-        <v>20</v>
+        <v>130</v>
       </c>
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.25">
@@ -5465,13 +5474,13 @@
         <v>127</v>
       </c>
       <c r="B319" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="C319" t="b">
         <v>0</v>
       </c>
       <c r="D319" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.25">
@@ -5479,7 +5488,7 @@
         <v>127</v>
       </c>
       <c r="B320" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C320" t="b">
         <v>0</v>
@@ -5493,7 +5502,7 @@
         <v>127</v>
       </c>
       <c r="B321" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C321" t="b">
         <v>0</v>
@@ -5507,7 +5516,7 @@
         <v>127</v>
       </c>
       <c r="B322" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C322" t="b">
         <v>0</v>
@@ -5521,13 +5530,13 @@
         <v>127</v>
       </c>
       <c r="B323" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C323" t="b">
         <v>0</v>
       </c>
       <c r="D323" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="324" spans="1:4" x14ac:dyDescent="0.25">
@@ -5535,13 +5544,13 @@
         <v>127</v>
       </c>
       <c r="B324" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C324" t="b">
         <v>0</v>
       </c>
       <c r="D324" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.25">
@@ -5549,13 +5558,13 @@
         <v>127</v>
       </c>
       <c r="B325" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="C325" t="b">
         <v>0</v>
       </c>
       <c r="D325" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="326" spans="1:4" x14ac:dyDescent="0.25">
@@ -5563,27 +5572,27 @@
         <v>127</v>
       </c>
       <c r="B326" t="s">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="C326" t="b">
         <v>0</v>
       </c>
       <c r="D326" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="327" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B327" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C327" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D327" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.25">
@@ -5591,10 +5600,10 @@
         <v>131</v>
       </c>
       <c r="B328" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C328" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D328" t="s">
         <v>6</v>
@@ -5605,10 +5614,10 @@
         <v>131</v>
       </c>
       <c r="B329" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="C329" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D329" t="s">
         <v>6</v>
@@ -5619,7 +5628,7 @@
         <v>131</v>
       </c>
       <c r="B330" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C330" t="b">
         <v>1</v>
@@ -5633,13 +5642,13 @@
         <v>131</v>
       </c>
       <c r="B331" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C331" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D331" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.25">
@@ -5647,13 +5656,13 @@
         <v>131</v>
       </c>
       <c r="B332" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C332" t="b">
         <v>0</v>
       </c>
       <c r="D332" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
@@ -5661,7 +5670,7 @@
         <v>131</v>
       </c>
       <c r="B333" t="s">
-        <v>116</v>
+        <v>38</v>
       </c>
       <c r="C333" t="b">
         <v>0</v>
@@ -5672,13 +5681,13 @@
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B334" t="s">
-        <v>5</v>
+        <v>116</v>
       </c>
       <c r="C334" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D334" t="s">
         <v>6</v>
@@ -5689,10 +5698,10 @@
         <v>132</v>
       </c>
       <c r="B335" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C335" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D335" t="s">
         <v>6</v>
@@ -5703,13 +5712,13 @@
         <v>132</v>
       </c>
       <c r="B336" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C336" t="b">
         <v>0</v>
       </c>
       <c r="D336" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="337" spans="1:4" x14ac:dyDescent="0.25">
@@ -5717,13 +5726,13 @@
         <v>132</v>
       </c>
       <c r="B337" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C337" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D337" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.25">
@@ -5731,10 +5740,10 @@
         <v>132</v>
       </c>
       <c r="B338" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C338" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D338" t="s">
         <v>6</v>
@@ -5745,7 +5754,7 @@
         <v>132</v>
       </c>
       <c r="B339" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C339" t="b">
         <v>0</v>
@@ -5759,10 +5768,10 @@
         <v>132</v>
       </c>
       <c r="B340" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C340" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D340" t="s">
         <v>6</v>
@@ -5773,13 +5782,13 @@
         <v>132</v>
       </c>
       <c r="B341" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C341" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D341" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.25">
@@ -5787,13 +5796,13 @@
         <v>132</v>
       </c>
       <c r="B342" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C342" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D342" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
@@ -5801,10 +5810,10 @@
         <v>132</v>
       </c>
       <c r="B343" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C343" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D343" t="s">
         <v>6</v>
@@ -5815,10 +5824,10 @@
         <v>132</v>
       </c>
       <c r="B344" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C344" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D344" t="s">
         <v>6</v>
@@ -5829,7 +5838,7 @@
         <v>132</v>
       </c>
       <c r="B345" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C345" t="b">
         <v>1</v>
@@ -5843,10 +5852,10 @@
         <v>132</v>
       </c>
       <c r="B346" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C346" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D346" t="s">
         <v>6</v>
@@ -5857,13 +5866,13 @@
         <v>132</v>
       </c>
       <c r="B347" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C347" t="b">
         <v>0</v>
       </c>
       <c r="D347" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.25">
@@ -5871,13 +5880,13 @@
         <v>132</v>
       </c>
       <c r="B348" t="s">
-        <v>133</v>
+        <v>61</v>
       </c>
       <c r="C348" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D348" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="349" spans="1:4" x14ac:dyDescent="0.25">
@@ -5885,13 +5894,13 @@
         <v>132</v>
       </c>
       <c r="B349" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C349" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D349" t="s">
-        <v>135</v>
+        <v>51</v>
       </c>
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.25">
@@ -5899,13 +5908,13 @@
         <v>132</v>
       </c>
       <c r="B350" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C350" t="b">
         <v>0</v>
       </c>
       <c r="D350" t="s">
-        <v>9</v>
+        <v>135</v>
       </c>
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
@@ -5913,13 +5922,13 @@
         <v>132</v>
       </c>
       <c r="B351" t="s">
-        <v>19</v>
+        <v>136</v>
       </c>
       <c r="C351" t="b">
         <v>0</v>
       </c>
       <c r="D351" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.25">
@@ -5927,13 +5936,13 @@
         <v>132</v>
       </c>
       <c r="B352" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C352" t="b">
         <v>0</v>
       </c>
       <c r="D352" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
@@ -5941,13 +5950,13 @@
         <v>132</v>
       </c>
       <c r="B353" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C353" t="b">
         <v>0</v>
       </c>
       <c r="D353" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
@@ -5955,27 +5964,27 @@
         <v>132</v>
       </c>
       <c r="B354" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C354" t="b">
         <v>0</v>
       </c>
       <c r="D354" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="355" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B355" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C355" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D355" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
@@ -5983,10 +5992,10 @@
         <v>137</v>
       </c>
       <c r="B356" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C356" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D356" t="s">
         <v>6</v>
@@ -5997,13 +6006,13 @@
         <v>137</v>
       </c>
       <c r="B357" t="s">
-        <v>133</v>
+        <v>12</v>
       </c>
       <c r="C357" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D357" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.25">
@@ -6011,10 +6020,10 @@
         <v>137</v>
       </c>
       <c r="B358" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C358" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D358" t="s">
         <v>51</v>
@@ -6025,13 +6034,13 @@
         <v>137</v>
       </c>
       <c r="B359" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C359" t="b">
         <v>0</v>
       </c>
       <c r="D359" t="s">
-        <v>140</v>
+        <v>51</v>
       </c>
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.25">
@@ -6039,13 +6048,13 @@
         <v>137</v>
       </c>
       <c r="B360" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C360" t="b">
         <v>0</v>
       </c>
       <c r="D360" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.25">
@@ -6053,13 +6062,13 @@
         <v>137</v>
       </c>
       <c r="B361" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C361" t="b">
         <v>0</v>
       </c>
       <c r="D361" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.25">
@@ -6067,27 +6076,27 @@
         <v>137</v>
       </c>
       <c r="B362" t="s">
-        <v>32</v>
+        <v>143</v>
       </c>
       <c r="C362" t="b">
         <v>0</v>
       </c>
       <c r="D362" t="s">
-        <v>33</v>
+        <v>144</v>
       </c>
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B363" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C363" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D363" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.25">
@@ -6095,10 +6104,10 @@
         <v>145</v>
       </c>
       <c r="B364" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C364" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D364" t="s">
         <v>6</v>
@@ -6109,13 +6118,13 @@
         <v>145</v>
       </c>
       <c r="B365" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C365" t="b">
         <v>0</v>
       </c>
       <c r="D365" t="s">
-        <v>148</v>
+        <v>6</v>
       </c>
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.25">
@@ -6123,27 +6132,27 @@
         <v>145</v>
       </c>
       <c r="B366" t="s">
-        <v>32</v>
+        <v>147</v>
       </c>
       <c r="C366" t="b">
         <v>0</v>
       </c>
       <c r="D366" t="s">
-        <v>33</v>
+        <v>148</v>
       </c>
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B367" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C367" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D367" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
@@ -6151,10 +6160,10 @@
         <v>149</v>
       </c>
       <c r="B368" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C368" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D368" t="s">
         <v>6</v>
@@ -6165,13 +6174,13 @@
         <v>149</v>
       </c>
       <c r="B369" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C369" t="b">
         <v>0</v>
       </c>
       <c r="D369" t="s">
-        <v>150</v>
+        <v>6</v>
       </c>
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
@@ -6179,13 +6188,13 @@
         <v>149</v>
       </c>
       <c r="B370" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C370" t="b">
         <v>0</v>
       </c>
       <c r="D370" t="s">
-        <v>9</v>
+        <v>150</v>
       </c>
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
@@ -6193,35 +6202,35 @@
         <v>149</v>
       </c>
       <c r="B371" t="s">
-        <v>32</v>
+        <v>151</v>
       </c>
       <c r="C371" t="b">
         <v>0</v>
       </c>
       <c r="D371" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B372" t="s">
-        <v>153</v>
+        <v>32</v>
       </c>
       <c r="C372" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D372" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B373" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C373" t="b">
         <v>1</v>
@@ -6232,10 +6241,10 @@
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B374" t="s">
-        <v>5</v>
+        <v>155</v>
       </c>
       <c r="C374" t="b">
         <v>1</v>
@@ -6249,10 +6258,10 @@
         <v>156</v>
       </c>
       <c r="B375" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C375" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D375" t="s">
         <v>6</v>
@@ -6263,150 +6272,150 @@
         <v>156</v>
       </c>
       <c r="B376" t="s">
-        <v>32</v>
+        <v>146</v>
       </c>
       <c r="C376" t="b">
         <v>0</v>
       </c>
       <c r="D376" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
+        <v>156</v>
+      </c>
+      <c r="B377" t="s">
+        <v>147</v>
+      </c>
+      <c r="C377" t="b">
+        <v>0</v>
+      </c>
+      <c r="D377" t="s">
         <v>157</v>
-      </c>
-      <c r="B377" t="s">
-        <v>5</v>
-      </c>
-      <c r="C377" t="b">
-        <v>1</v>
-      </c>
-      <c r="D377" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="378" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B378" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C378" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D378" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B379" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C379" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D379" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B380" t="s">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="C380" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D380" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B381" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C381" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D381" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="382" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B382" t="s">
-        <v>34</v>
+        <v>161</v>
       </c>
       <c r="C382" t="b">
         <v>0</v>
       </c>
       <c r="D382" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B383" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C383" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D383" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="384" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B384" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="C384" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D384" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B385" t="s">
-        <v>160</v>
+        <v>34</v>
       </c>
       <c r="C385" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D385" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B386" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C386" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D386" t="s">
         <v>6</v>
@@ -6414,13 +6423,13 @@
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B387" t="s">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="C387" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D387" t="s">
         <v>6</v>
@@ -6428,10 +6437,10 @@
     </row>
     <row r="388" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B388" t="s">
-        <v>10</v>
+        <v>163</v>
       </c>
       <c r="C388" t="b">
         <v>1</v>
@@ -6442,13 +6451,13 @@
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B389" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C389" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D389" t="s">
         <v>6</v>
@@ -6456,10 +6465,10 @@
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B390" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="C390" t="b">
         <v>0</v>
@@ -6470,7 +6479,7 @@
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B391" t="s">
         <v>10</v>
@@ -6484,7 +6493,7 @@
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B392" t="s">
         <v>99</v>
@@ -6498,7 +6507,7 @@
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B393" t="s">
         <v>12</v>
@@ -6512,10 +6521,10 @@
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B394" t="s">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="C394" t="b">
         <v>1</v>
@@ -6526,10 +6535,10 @@
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B395" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C395" t="b">
         <v>1</v>
@@ -6540,10 +6549,10 @@
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B396" t="s">
-        <v>115</v>
+        <v>12</v>
       </c>
       <c r="C396" t="b">
         <v>0</v>
@@ -6554,10 +6563,10 @@
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B397" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C397" t="b">
         <v>1</v>
@@ -6568,7 +6577,7 @@
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B398" t="s">
         <v>97</v>
@@ -6582,7 +6591,7 @@
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B399" t="s">
         <v>115</v>
@@ -6596,7 +6605,7 @@
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B400" t="s">
         <v>99</v>
@@ -6610,7 +6619,7 @@
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B401" t="s">
         <v>97</v>
@@ -6624,7 +6633,7 @@
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B402" t="s">
         <v>115</v>
@@ -6638,7 +6647,7 @@
     </row>
     <row r="403" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B403" t="s">
         <v>99</v>
@@ -6652,13 +6661,13 @@
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B404" t="s">
-        <v>167</v>
+        <v>97</v>
       </c>
       <c r="C404" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D404" t="s">
         <v>6</v>
@@ -6666,10 +6675,10 @@
     </row>
     <row r="405" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B405" t="s">
-        <v>7</v>
+        <v>115</v>
       </c>
       <c r="C405" t="b">
         <v>0</v>
@@ -6680,52 +6689,52 @@
     </row>
     <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B406" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="C406" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D406" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B407" t="s">
-        <v>32</v>
+        <v>170</v>
       </c>
       <c r="C407" t="b">
         <v>0</v>
       </c>
       <c r="D407" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B408" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="C408" t="b">
         <v>0</v>
       </c>
       <c r="D408" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B409" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C409" t="b">
         <v>0</v>
@@ -6736,66 +6745,66 @@
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B410" t="s">
-        <v>169</v>
+        <v>32</v>
       </c>
       <c r="C410" t="b">
         <v>0</v>
       </c>
       <c r="D410" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B411" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C411" t="b">
         <v>0</v>
       </c>
       <c r="D411" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B412" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C412" t="b">
         <v>0</v>
       </c>
       <c r="D412" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B413" t="s">
-        <v>34</v>
+        <v>172</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
       </c>
       <c r="D413" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B414" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C414" t="b">
         <v>0</v>
@@ -6806,38 +6815,38 @@
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B415" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="C415" t="b">
         <v>0</v>
       </c>
       <c r="D415" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B416" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C416" t="b">
         <v>0</v>
       </c>
       <c r="D416" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B417" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C417" t="b">
         <v>0</v>
@@ -6848,38 +6857,38 @@
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B418" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="C418" t="b">
         <v>0</v>
       </c>
       <c r="D418" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B419" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="C419" t="b">
         <v>0</v>
       </c>
       <c r="D419" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B420" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C420" t="b">
         <v>0</v>
@@ -6890,49 +6899,49 @@
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B421" t="s">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="C421" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D421" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B422" t="s">
-        <v>115</v>
+        <v>34</v>
       </c>
       <c r="C422" t="b">
         <v>0</v>
       </c>
       <c r="D422" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B423" t="s">
-        <v>172</v>
+        <v>31</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
       </c>
       <c r="D423" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B424" t="s">
         <v>97</v>
@@ -6946,7 +6955,7 @@
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B425" t="s">
         <v>115</v>
@@ -6960,10 +6969,10 @@
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B426" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C426" t="b">
         <v>0</v>
@@ -6974,13 +6983,13 @@
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B427" t="s">
-        <v>174</v>
+        <v>97</v>
       </c>
       <c r="C427" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D427" t="s">
         <v>6</v>
@@ -6988,13 +6997,13 @@
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B428" t="s">
-        <v>176</v>
+        <v>115</v>
       </c>
       <c r="C428" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D428" t="s">
         <v>6</v>
@@ -7002,13 +7011,13 @@
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
+        <v>176</v>
+      </c>
+      <c r="B429" t="s">
         <v>175</v>
       </c>
-      <c r="B429" t="s">
-        <v>10</v>
-      </c>
       <c r="C429" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D429" t="s">
         <v>6</v>
@@ -7016,10 +7025,10 @@
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B430" t="s">
-        <v>12</v>
+        <v>177</v>
       </c>
       <c r="C430" t="b">
         <v>0</v>
@@ -7030,58 +7039,58 @@
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B431" t="s">
-        <v>32</v>
+        <v>179</v>
       </c>
       <c r="C431" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D431" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B432" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C432" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D432" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B433" t="s">
-        <v>177</v>
+        <v>12</v>
       </c>
       <c r="C433" t="b">
         <v>0</v>
       </c>
       <c r="D433" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B434" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C434" t="b">
         <v>0</v>
       </c>
       <c r="D434" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
@@ -7089,13 +7098,13 @@
         <v>178</v>
       </c>
       <c r="B435" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="C435" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D435" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
@@ -7103,13 +7112,13 @@
         <v>178</v>
       </c>
       <c r="B436" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C436" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D436" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
@@ -7117,10 +7126,10 @@
         <v>178</v>
       </c>
       <c r="B437" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="C437" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D437" t="s">
         <v>6</v>
@@ -7128,13 +7137,13 @@
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B438" t="s">
-        <v>12</v>
+        <v>182</v>
       </c>
       <c r="C438" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D438" t="s">
         <v>6</v>
@@ -7142,86 +7151,86 @@
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B439" t="s">
-        <v>32</v>
+        <v>179</v>
       </c>
       <c r="C439" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D439" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="440" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B440" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C440" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D440" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="441" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B441" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="C441" t="b">
         <v>0</v>
       </c>
       <c r="D441" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B442" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C442" t="b">
         <v>0</v>
       </c>
       <c r="D442" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="443" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="B443" t="s">
-        <v>180</v>
+        <v>8</v>
       </c>
       <c r="C443" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D443" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="444" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="B444" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="C444" t="b">
         <v>0</v>
       </c>
       <c r="D444" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="445" spans="1:4" x14ac:dyDescent="0.25">
@@ -7229,38 +7238,38 @@
         <v>181</v>
       </c>
       <c r="B445" t="s">
-        <v>182</v>
+        <v>38</v>
       </c>
       <c r="C445" t="b">
         <v>0</v>
       </c>
       <c r="D445" t="s">
-        <v>183</v>
+        <v>6</v>
       </c>
     </row>
     <row r="446" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
-        <v>181</v>
+        <v>84</v>
       </c>
       <c r="B446" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C446" t="b">
         <v>1</v>
       </c>
       <c r="D446" t="s">
-        <v>185</v>
+        <v>6</v>
       </c>
     </row>
     <row r="447" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
-        <v>186</v>
+        <v>84</v>
       </c>
       <c r="B447" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C447" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D447" t="s">
         <v>6</v>
@@ -7268,38 +7277,38 @@
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
+        <v>184</v>
+      </c>
+      <c r="B448" t="s">
+        <v>185</v>
+      </c>
+      <c r="C448" t="b">
+        <v>0</v>
+      </c>
+      <c r="D448" t="s">
         <v>186</v>
-      </c>
-      <c r="B448" t="s">
-        <v>187</v>
-      </c>
-      <c r="C448" t="b">
-        <v>1</v>
-      </c>
-      <c r="D448" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
+        <v>184</v>
+      </c>
+      <c r="B449" t="s">
+        <v>187</v>
+      </c>
+      <c r="C449" t="b">
+        <v>1</v>
+      </c>
+      <c r="D449" t="s">
         <v>188</v>
-      </c>
-      <c r="B449" t="s">
-        <v>5</v>
-      </c>
-      <c r="C449" t="b">
-        <v>1</v>
-      </c>
-      <c r="D449" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B450" t="s">
-        <v>187</v>
+        <v>5</v>
       </c>
       <c r="C450" t="b">
         <v>1</v>
@@ -7313,7 +7322,7 @@
         <v>189</v>
       </c>
       <c r="B451" t="s">
-        <v>97</v>
+        <v>190</v>
       </c>
       <c r="C451" t="b">
         <v>1</v>
@@ -7324,10 +7333,10 @@
     </row>
     <row r="452" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B452" t="s">
-        <v>190</v>
+        <v>5</v>
       </c>
       <c r="C452" t="b">
         <v>1</v>
@@ -7341,7 +7350,7 @@
         <v>191</v>
       </c>
       <c r="B453" t="s">
-        <v>97</v>
+        <v>190</v>
       </c>
       <c r="C453" t="b">
         <v>1</v>
@@ -7352,10 +7361,10 @@
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B454" t="s">
-        <v>192</v>
+        <v>97</v>
       </c>
       <c r="C454" t="b">
         <v>1</v>
@@ -7366,10 +7375,10 @@
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
+        <v>192</v>
+      </c>
+      <c r="B455" t="s">
         <v>193</v>
-      </c>
-      <c r="B455" t="s">
-        <v>5</v>
       </c>
       <c r="C455" t="b">
         <v>1</v>
@@ -7383,7 +7392,7 @@
         <v>194</v>
       </c>
       <c r="B456" t="s">
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="C456" t="b">
         <v>1</v>
@@ -7394,10 +7403,10 @@
     </row>
     <row r="457" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
+        <v>194</v>
+      </c>
+      <c r="B457" t="s">
         <v>195</v>
-      </c>
-      <c r="B457" t="s">
-        <v>196</v>
       </c>
       <c r="C457" t="b">
         <v>1</v>
@@ -7408,7 +7417,7 @@
     </row>
     <row r="458" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B458" t="s">
         <v>5</v>
@@ -7425,10 +7434,10 @@
         <v>197</v>
       </c>
       <c r="B459" t="s">
-        <v>198</v>
+        <v>5</v>
       </c>
       <c r="C459" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D459" t="s">
         <v>6</v>
@@ -7436,10 +7445,10 @@
     </row>
     <row r="460" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
+        <v>198</v>
+      </c>
+      <c r="B460" t="s">
         <v>199</v>
-      </c>
-      <c r="B460" t="s">
-        <v>5</v>
       </c>
       <c r="C460" t="b">
         <v>1</v>
@@ -7450,13 +7459,13 @@
     </row>
     <row r="461" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B461" t="s">
-        <v>198</v>
+        <v>5</v>
       </c>
       <c r="C461" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D461" t="s">
         <v>6</v>
@@ -7467,10 +7476,10 @@
         <v>200</v>
       </c>
       <c r="B462" t="s">
-        <v>5</v>
+        <v>201</v>
       </c>
       <c r="C462" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D462" t="s">
         <v>6</v>
@@ -7478,13 +7487,13 @@
     </row>
     <row r="463" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B463" t="s">
-        <v>198</v>
+        <v>5</v>
       </c>
       <c r="C463" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D463" t="s">
         <v>6</v>
@@ -7492,13 +7501,13 @@
     </row>
     <row r="464" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
+        <v>202</v>
+      </c>
+      <c r="B464" t="s">
         <v>201</v>
       </c>
-      <c r="B464" t="s">
-        <v>5</v>
-      </c>
       <c r="C464" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D464" t="s">
         <v>6</v>
@@ -7506,13 +7515,13 @@
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B465" t="s">
-        <v>198</v>
+        <v>5</v>
       </c>
       <c r="C465" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D465" t="s">
         <v>6</v>
@@ -7520,13 +7529,13 @@
     </row>
     <row r="466" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B466" t="s">
-        <v>5</v>
+        <v>201</v>
       </c>
       <c r="C466" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D466" t="s">
         <v>6</v>
@@ -7534,13 +7543,13 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B467" t="s">
         <v>5</v>
       </c>
       <c r="C467" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D467" t="s">
         <v>6</v>
@@ -7548,10 +7557,10 @@
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B468" t="s">
-        <v>179</v>
+        <v>201</v>
       </c>
       <c r="C468" t="b">
         <v>0</v>
@@ -7562,13 +7571,13 @@
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B469" t="s">
-        <v>176</v>
+        <v>5</v>
       </c>
       <c r="C469" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D469" t="s">
         <v>6</v>
@@ -7576,13 +7585,13 @@
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B470" t="s">
-        <v>204</v>
+        <v>5</v>
       </c>
       <c r="C470" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D470" t="s">
         <v>6</v>
@@ -7590,10 +7599,10 @@
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B471" t="s">
-        <v>12</v>
+        <v>182</v>
       </c>
       <c r="C471" t="b">
         <v>0</v>
@@ -7604,13 +7613,13 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B472" t="s">
-        <v>5</v>
+        <v>179</v>
       </c>
       <c r="C472" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D472" t="s">
         <v>6</v>
@@ -7618,13 +7627,13 @@
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B473" t="s">
-        <v>7</v>
+        <v>207</v>
       </c>
       <c r="C473" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D473" t="s">
         <v>6</v>
@@ -7632,24 +7641,24 @@
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B474" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C474" t="b">
         <v>0</v>
       </c>
       <c r="D474" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="475" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B475" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C475" t="b">
         <v>1</v>
@@ -7660,10 +7669,10 @@
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B476" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C476" t="b">
         <v>0</v>
@@ -7674,24 +7683,24 @@
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B477" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C477" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D477" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B478" t="s">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="C478" t="b">
         <v>1</v>
@@ -7702,24 +7711,24 @@
     </row>
     <row r="479" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B479" t="s">
-        <v>46</v>
+        <v>11</v>
       </c>
       <c r="C479" t="b">
         <v>0</v>
       </c>
       <c r="D479" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="480" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B480" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C480" t="b">
         <v>1</v>
@@ -7730,13 +7739,13 @@
     </row>
     <row r="481" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B481" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="C481" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D481" t="s">
         <v>6</v>
@@ -7744,24 +7753,24 @@
     </row>
     <row r="482" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A482" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B482" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C482" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D482" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="483" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A483" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B483" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="C483" t="b">
         <v>1</v>
@@ -7772,57 +7781,99 @@
     </row>
     <row r="484" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A484" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B484" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="C484" t="b">
         <v>0</v>
       </c>
       <c r="D484" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="485" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A485" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B485" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C485" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D485" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="486" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A486" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B486" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="C486" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D486" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="487" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A487" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B487" t="s">
+        <v>19</v>
+      </c>
+      <c r="C487" t="b">
+        <v>0</v>
+      </c>
+      <c r="D487" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="488" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A488" t="s">
+        <v>208</v>
+      </c>
+      <c r="B488" t="s">
+        <v>31</v>
+      </c>
+      <c r="C488" t="b">
+        <v>0</v>
+      </c>
+      <c r="D488" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="489" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A489" t="s">
+        <v>208</v>
+      </c>
+      <c r="B489" t="s">
+        <v>32</v>
+      </c>
+      <c r="C489" t="b">
+        <v>0</v>
+      </c>
+      <c r="D489" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="490" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A490" t="s">
+        <v>208</v>
+      </c>
+      <c r="B490" t="s">
         <v>34</v>
       </c>
-      <c r="C487" t="b">
-        <v>0</v>
-      </c>
-      <c r="D487" t="s">
+      <c r="C490" t="b">
+        <v>0</v>
+      </c>
+      <c r="D490" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>